<commit_message>
update md process files
</commit_message>
<xml_diff>
--- a/resources/metadata_process_scripts/sources/catalog.xlsx
+++ b/resources/metadata_process_scripts/sources/catalog.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12280" uniqueCount="2449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12304" uniqueCount="2447">
   <si>
     <t>ds:DatName</t>
   </si>
@@ -7302,22 +7302,16 @@
     <t>2018-SmartUnitn2-additional_material-questionnaire</t>
   </si>
   <si>
+    <t>Dataset paper and data collection methodology</t>
+  </si>
+  <si>
     <t>https://drive.google.com/file/d/1yY8RNaWO_eh4-UnXHkL2jpZld2739K3K/view?usp=share_link</t>
   </si>
   <si>
-    <t>2018-SmartUnitn2-technical_report</t>
-  </si>
-  <si>
-    <t>2022_WeNet_Diversity1_Technical-Report(2020-2021)</t>
-  </si>
-  <si>
-    <t>2021-Chatbot1-technical_report</t>
-  </si>
-  <si>
-    <t>2022_LivePeople_Chatbot2_Data_Descriptor</t>
-  </si>
-  <si>
-    <t>Big-Thick Data generation via reference and personal context unification</t>
+    <t>https://arxiv.org/abs/2502.03347</t>
+  </si>
+  <si>
+    <t>Dataset technical report</t>
   </si>
   <si>
     <t>https://drive.google.com/file/d/1mSIBHgKJBw07crEjMTYEi3ylpPL-62fB/view?usp=sharing</t>
@@ -53947,16 +53941,16 @@
         <v>2427</v>
       </c>
       <c r="AG2" s="4" t="s">
-        <v>2428</v>
+        <v>2429</v>
       </c>
       <c r="AH2" t="s">
         <v>1031</v>
       </c>
       <c r="AI2" t="s">
-        <v>2429</v>
+        <v>2431</v>
       </c>
       <c r="AJ2" s="4" t="s">
-        <v>2434</v>
+        <v>2432</v>
       </c>
       <c r="AK2" t="s">
         <v>1031</v>
@@ -53968,10 +53962,10 @@
         <v>1855</v>
       </c>
       <c r="AN2" t="s">
-        <v>2439</v>
+        <v>2437</v>
       </c>
       <c r="AO2" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP2" t="b">
         <v>1</v>
@@ -54057,10 +54051,10 @@
         <v>1855</v>
       </c>
       <c r="AN3" t="s">
-        <v>2440</v>
+        <v>2438</v>
       </c>
       <c r="AO3" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP3" t="b">
         <v>1</v>
@@ -54142,11 +54136,20 @@
       <c r="AE4" t="s">
         <v>657</v>
       </c>
+      <c r="AF4" t="s">
+        <v>2428</v>
+      </c>
+      <c r="AG4" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>1031</v>
+      </c>
       <c r="AI4" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="AJ4" s="4" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="AK4" t="s">
         <v>1031</v>
@@ -54158,10 +54161,10 @@
         <v>1856</v>
       </c>
       <c r="AN4" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="AO4" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP4" t="b">
         <v>1</v>
@@ -54243,11 +54246,20 @@
       <c r="AE5" t="s">
         <v>657</v>
       </c>
+      <c r="AF5" t="s">
+        <v>2428</v>
+      </c>
+      <c r="AG5" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>1031</v>
+      </c>
       <c r="AI5" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="AJ5" s="4" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="AK5" t="s">
         <v>1031</v>
@@ -54259,10 +54271,10 @@
         <v>1857</v>
       </c>
       <c r="AN5" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="AO5" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP5" t="b">
         <v>1</v>
@@ -54347,11 +54359,20 @@
       <c r="AE6" t="s">
         <v>657</v>
       </c>
+      <c r="AF6" t="s">
+        <v>2428</v>
+      </c>
+      <c r="AG6" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>1031</v>
+      </c>
       <c r="AI6" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="AJ6" s="4" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="AK6" t="s">
         <v>1031</v>
@@ -54363,10 +54384,10 @@
         <v>1858</v>
       </c>
       <c r="AN6" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="AO6" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP6" t="b">
         <v>1</v>
@@ -54448,11 +54469,20 @@
       <c r="AE7" t="s">
         <v>657</v>
       </c>
+      <c r="AF7" t="s">
+        <v>2428</v>
+      </c>
+      <c r="AG7" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>1031</v>
+      </c>
       <c r="AI7" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="AJ7" s="4" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="AK7" t="s">
         <v>1031</v>
@@ -54464,10 +54494,10 @@
         <v>1859</v>
       </c>
       <c r="AN7" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="AO7" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP7" t="b">
         <v>1</v>
@@ -54549,11 +54579,20 @@
       <c r="AE8" t="s">
         <v>657</v>
       </c>
+      <c r="AF8" t="s">
+        <v>2428</v>
+      </c>
+      <c r="AG8" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>1031</v>
+      </c>
       <c r="AI8" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="AJ8" s="4" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="AK8" t="s">
         <v>1031</v>
@@ -54565,10 +54604,10 @@
         <v>1860</v>
       </c>
       <c r="AN8" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="AO8" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP8" t="b">
         <v>1</v>
@@ -54650,11 +54689,20 @@
       <c r="AE9" t="s">
         <v>657</v>
       </c>
+      <c r="AF9" t="s">
+        <v>2428</v>
+      </c>
+      <c r="AG9" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>1031</v>
+      </c>
       <c r="AI9" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="AJ9" s="4" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="AK9" t="s">
         <v>1031</v>
@@ -54666,10 +54714,10 @@
         <v>1861</v>
       </c>
       <c r="AN9" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="AO9" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP9" t="b">
         <v>1</v>
@@ -54754,11 +54802,20 @@
       <c r="AE10" t="s">
         <v>657</v>
       </c>
+      <c r="AF10" t="s">
+        <v>2428</v>
+      </c>
+      <c r="AG10" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>1031</v>
+      </c>
       <c r="AI10" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="AJ10" s="4" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="AK10" t="s">
         <v>1031</v>
@@ -54770,10 +54827,10 @@
         <v>1855</v>
       </c>
       <c r="AN10" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="AO10" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP10" t="b">
         <v>1</v>
@@ -54855,11 +54912,20 @@
       <c r="AE11" t="s">
         <v>657</v>
       </c>
+      <c r="AF11" t="s">
+        <v>2428</v>
+      </c>
+      <c r="AG11" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>1031</v>
+      </c>
       <c r="AI11" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="AJ11" s="4" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
       <c r="AK11" t="s">
         <v>1031</v>
@@ -54871,10 +54937,10 @@
         <v>1862</v>
       </c>
       <c r="AN11" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="AO11" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP11" t="b">
         <v>1</v>
@@ -54957,7 +55023,7 @@
         <v>2431</v>
       </c>
       <c r="AJ12" s="4" t="s">
-        <v>2436</v>
+        <v>2434</v>
       </c>
       <c r="AK12" t="s">
         <v>1031</v>
@@ -54969,10 +55035,10 @@
         <v>1857</v>
       </c>
       <c r="AN12" t="s">
-        <v>2442</v>
+        <v>2440</v>
       </c>
       <c r="AO12" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP12" t="b">
         <v>1</v>
@@ -55058,7 +55124,7 @@
         <v>2431</v>
       </c>
       <c r="AJ13" s="4" t="s">
-        <v>2436</v>
+        <v>2434</v>
       </c>
       <c r="AK13" t="s">
         <v>1031</v>
@@ -55070,10 +55136,10 @@
         <v>1858</v>
       </c>
       <c r="AN13" t="s">
-        <v>2442</v>
+        <v>2440</v>
       </c>
       <c r="AO13" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP13" t="b">
         <v>1</v>
@@ -55156,7 +55222,7 @@
         <v>2431</v>
       </c>
       <c r="AJ14" s="4" t="s">
-        <v>2436</v>
+        <v>2434</v>
       </c>
       <c r="AK14" t="s">
         <v>1031</v>
@@ -55168,10 +55234,10 @@
         <v>1860</v>
       </c>
       <c r="AN14" t="s">
-        <v>2442</v>
+        <v>2440</v>
       </c>
       <c r="AO14" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP14" t="b">
         <v>1</v>
@@ -55257,7 +55323,7 @@
         <v>2431</v>
       </c>
       <c r="AJ15" s="4" t="s">
-        <v>2436</v>
+        <v>2434</v>
       </c>
       <c r="AK15" t="s">
         <v>1031</v>
@@ -55269,10 +55335,10 @@
         <v>1855</v>
       </c>
       <c r="AN15" t="s">
-        <v>2442</v>
+        <v>2440</v>
       </c>
       <c r="AO15" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP15" t="b">
         <v>1</v>
@@ -55355,7 +55421,7 @@
         <v>2431</v>
       </c>
       <c r="AJ16" s="4" t="s">
-        <v>2436</v>
+        <v>2434</v>
       </c>
       <c r="AK16" t="s">
         <v>1031</v>
@@ -55367,10 +55433,10 @@
         <v>1862</v>
       </c>
       <c r="AN16" t="s">
-        <v>2442</v>
+        <v>2440</v>
       </c>
       <c r="AO16" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP16" t="b">
         <v>1</v>
@@ -55450,10 +55516,10 @@
         <v>657</v>
       </c>
       <c r="AI17" t="s">
-        <v>2432</v>
+        <v>2431</v>
       </c>
       <c r="AJ17" s="4" t="s">
-        <v>2437</v>
+        <v>2435</v>
       </c>
       <c r="AK17" t="s">
         <v>1031</v>
@@ -55465,10 +55531,10 @@
         <v>1857</v>
       </c>
       <c r="AN17" t="s">
-        <v>2443</v>
+        <v>2441</v>
       </c>
       <c r="AO17" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP17" t="b">
         <v>1</v>
@@ -55551,10 +55617,10 @@
         <v>657</v>
       </c>
       <c r="AI18" t="s">
-        <v>2432</v>
+        <v>2431</v>
       </c>
       <c r="AJ18" s="4" t="s">
-        <v>2437</v>
+        <v>2435</v>
       </c>
       <c r="AK18" t="s">
         <v>1031</v>
@@ -55566,10 +55632,10 @@
         <v>1858</v>
       </c>
       <c r="AN18" t="s">
-        <v>2443</v>
+        <v>2441</v>
       </c>
       <c r="AO18" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP18" t="b">
         <v>1</v>
@@ -55649,10 +55715,10 @@
         <v>657</v>
       </c>
       <c r="AI19" t="s">
-        <v>2432</v>
+        <v>2431</v>
       </c>
       <c r="AJ19" s="4" t="s">
-        <v>2437</v>
+        <v>2435</v>
       </c>
       <c r="AK19" t="s">
         <v>1031</v>
@@ -55664,10 +55730,10 @@
         <v>1860</v>
       </c>
       <c r="AN19" t="s">
-        <v>2443</v>
+        <v>2441</v>
       </c>
       <c r="AO19" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP19" t="b">
         <v>1</v>
@@ -55750,10 +55816,10 @@
         <v>657</v>
       </c>
       <c r="AI20" t="s">
-        <v>2432</v>
+        <v>2431</v>
       </c>
       <c r="AJ20" s="4" t="s">
-        <v>2437</v>
+        <v>2435</v>
       </c>
       <c r="AK20" t="s">
         <v>1031</v>
@@ -55765,10 +55831,10 @@
         <v>1855</v>
       </c>
       <c r="AN20" t="s">
-        <v>2443</v>
+        <v>2441</v>
       </c>
       <c r="AO20" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP20" t="b">
         <v>1</v>
@@ -55848,10 +55914,10 @@
         <v>657</v>
       </c>
       <c r="AI21" t="s">
-        <v>2432</v>
+        <v>2431</v>
       </c>
       <c r="AJ21" s="4" t="s">
-        <v>2437</v>
+        <v>2435</v>
       </c>
       <c r="AK21" t="s">
         <v>1031</v>
@@ -55863,10 +55929,10 @@
         <v>1862</v>
       </c>
       <c r="AN21" t="s">
-        <v>2443</v>
+        <v>2441</v>
       </c>
       <c r="AO21" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP21" t="b">
         <v>1</v>
@@ -55949,10 +56015,10 @@
         <v>1863</v>
       </c>
       <c r="AN22" t="s">
-        <v>2444</v>
+        <v>2442</v>
       </c>
       <c r="AO22" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP22" t="b">
         <v>1</v>
@@ -56038,10 +56104,10 @@
         <v>1864</v>
       </c>
       <c r="AN23" t="s">
-        <v>2444</v>
+        <v>2442</v>
       </c>
       <c r="AO23" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP23" t="b">
         <v>1</v>
@@ -56094,10 +56160,10 @@
         <v>1855</v>
       </c>
       <c r="AN24" t="s">
-        <v>2445</v>
+        <v>2443</v>
       </c>
       <c r="AO24" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP24" t="b">
         <v>0</v>
@@ -56141,10 +56207,10 @@
         <v>657</v>
       </c>
       <c r="AI25" t="s">
-        <v>2433</v>
+        <v>2431</v>
       </c>
       <c r="AJ25" s="4" t="s">
-        <v>2438</v>
+        <v>2436</v>
       </c>
       <c r="AK25" t="s">
         <v>1031</v>
@@ -56156,10 +56222,10 @@
         <v>1865</v>
       </c>
       <c r="AN25" t="s">
+        <v>2444</v>
+      </c>
+      <c r="AO25" t="s">
         <v>2446</v>
-      </c>
-      <c r="AO25" t="s">
-        <v>2448</v>
       </c>
       <c r="AP25" t="b">
         <v>1</v>
@@ -56239,10 +56305,10 @@
         <v>657</v>
       </c>
       <c r="AI26" t="s">
-        <v>2433</v>
+        <v>2431</v>
       </c>
       <c r="AJ26" s="4" t="s">
-        <v>2438</v>
+        <v>2436</v>
       </c>
       <c r="AK26" t="s">
         <v>1031</v>
@@ -56254,10 +56320,10 @@
         <v>1855</v>
       </c>
       <c r="AN26" t="s">
-        <v>2447</v>
+        <v>2445</v>
       </c>
       <c r="AO26" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="AP26" t="b">
         <v>1</v>
@@ -56272,56 +56338,64 @@
     <hyperlink ref="B3" r:id="rId5"/>
     <hyperlink ref="B4" r:id="rId6"/>
     <hyperlink ref="C4" r:id="rId7"/>
-    <hyperlink ref="AJ4" r:id="rId8"/>
-    <hyperlink ref="B5" r:id="rId9"/>
-    <hyperlink ref="C5" r:id="rId10"/>
-    <hyperlink ref="AJ5" r:id="rId11"/>
-    <hyperlink ref="B6" r:id="rId12"/>
-    <hyperlink ref="C6" r:id="rId13"/>
-    <hyperlink ref="AJ6" r:id="rId14"/>
-    <hyperlink ref="B7" r:id="rId15"/>
-    <hyperlink ref="C7" r:id="rId16"/>
-    <hyperlink ref="AJ7" r:id="rId17"/>
-    <hyperlink ref="B8" r:id="rId18"/>
-    <hyperlink ref="C8" r:id="rId19"/>
-    <hyperlink ref="AJ8" r:id="rId20"/>
-    <hyperlink ref="B9" r:id="rId21"/>
-    <hyperlink ref="C9" r:id="rId22"/>
-    <hyperlink ref="AJ9" r:id="rId23"/>
-    <hyperlink ref="B10" r:id="rId24"/>
-    <hyperlink ref="C10" r:id="rId25"/>
-    <hyperlink ref="AJ10" r:id="rId26"/>
-    <hyperlink ref="B11" r:id="rId27"/>
-    <hyperlink ref="C11" r:id="rId28"/>
-    <hyperlink ref="AJ11" r:id="rId29"/>
-    <hyperlink ref="B12" r:id="rId30"/>
-    <hyperlink ref="AJ12" r:id="rId31"/>
-    <hyperlink ref="B13" r:id="rId32"/>
-    <hyperlink ref="AJ13" r:id="rId33"/>
-    <hyperlink ref="B14" r:id="rId34"/>
-    <hyperlink ref="AJ14" r:id="rId35"/>
-    <hyperlink ref="B15" r:id="rId36"/>
-    <hyperlink ref="AJ15" r:id="rId37"/>
-    <hyperlink ref="B16" r:id="rId38"/>
-    <hyperlink ref="AJ16" r:id="rId39"/>
-    <hyperlink ref="B17" r:id="rId40"/>
-    <hyperlink ref="AJ17" r:id="rId41"/>
-    <hyperlink ref="B18" r:id="rId42"/>
-    <hyperlink ref="AJ18" r:id="rId43"/>
-    <hyperlink ref="B19" r:id="rId44"/>
-    <hyperlink ref="AJ19" r:id="rId45"/>
-    <hyperlink ref="B20" r:id="rId46"/>
-    <hyperlink ref="AJ20" r:id="rId47"/>
-    <hyperlink ref="B21" r:id="rId48"/>
-    <hyperlink ref="AJ21" r:id="rId49"/>
-    <hyperlink ref="B22" r:id="rId50"/>
-    <hyperlink ref="B23" r:id="rId51"/>
-    <hyperlink ref="B24" r:id="rId52"/>
-    <hyperlink ref="C24" r:id="rId53"/>
-    <hyperlink ref="B25" r:id="rId54"/>
-    <hyperlink ref="AJ25" r:id="rId55"/>
-    <hyperlink ref="B26" r:id="rId56"/>
-    <hyperlink ref="AJ26" r:id="rId57"/>
+    <hyperlink ref="AG4" r:id="rId8"/>
+    <hyperlink ref="AJ4" r:id="rId9"/>
+    <hyperlink ref="B5" r:id="rId10"/>
+    <hyperlink ref="C5" r:id="rId11"/>
+    <hyperlink ref="AG5" r:id="rId12"/>
+    <hyperlink ref="AJ5" r:id="rId13"/>
+    <hyperlink ref="B6" r:id="rId14"/>
+    <hyperlink ref="C6" r:id="rId15"/>
+    <hyperlink ref="AG6" r:id="rId16"/>
+    <hyperlink ref="AJ6" r:id="rId17"/>
+    <hyperlink ref="B7" r:id="rId18"/>
+    <hyperlink ref="C7" r:id="rId19"/>
+    <hyperlink ref="AG7" r:id="rId20"/>
+    <hyperlink ref="AJ7" r:id="rId21"/>
+    <hyperlink ref="B8" r:id="rId22"/>
+    <hyperlink ref="C8" r:id="rId23"/>
+    <hyperlink ref="AG8" r:id="rId24"/>
+    <hyperlink ref="AJ8" r:id="rId25"/>
+    <hyperlink ref="B9" r:id="rId26"/>
+    <hyperlink ref="C9" r:id="rId27"/>
+    <hyperlink ref="AG9" r:id="rId28"/>
+    <hyperlink ref="AJ9" r:id="rId29"/>
+    <hyperlink ref="B10" r:id="rId30"/>
+    <hyperlink ref="C10" r:id="rId31"/>
+    <hyperlink ref="AG10" r:id="rId32"/>
+    <hyperlink ref="AJ10" r:id="rId33"/>
+    <hyperlink ref="B11" r:id="rId34"/>
+    <hyperlink ref="C11" r:id="rId35"/>
+    <hyperlink ref="AG11" r:id="rId36"/>
+    <hyperlink ref="AJ11" r:id="rId37"/>
+    <hyperlink ref="B12" r:id="rId38"/>
+    <hyperlink ref="AJ12" r:id="rId39"/>
+    <hyperlink ref="B13" r:id="rId40"/>
+    <hyperlink ref="AJ13" r:id="rId41"/>
+    <hyperlink ref="B14" r:id="rId42"/>
+    <hyperlink ref="AJ14" r:id="rId43"/>
+    <hyperlink ref="B15" r:id="rId44"/>
+    <hyperlink ref="AJ15" r:id="rId45"/>
+    <hyperlink ref="B16" r:id="rId46"/>
+    <hyperlink ref="AJ16" r:id="rId47"/>
+    <hyperlink ref="B17" r:id="rId48"/>
+    <hyperlink ref="AJ17" r:id="rId49"/>
+    <hyperlink ref="B18" r:id="rId50"/>
+    <hyperlink ref="AJ18" r:id="rId51"/>
+    <hyperlink ref="B19" r:id="rId52"/>
+    <hyperlink ref="AJ19" r:id="rId53"/>
+    <hyperlink ref="B20" r:id="rId54"/>
+    <hyperlink ref="AJ20" r:id="rId55"/>
+    <hyperlink ref="B21" r:id="rId56"/>
+    <hyperlink ref="AJ21" r:id="rId57"/>
+    <hyperlink ref="B22" r:id="rId58"/>
+    <hyperlink ref="B23" r:id="rId59"/>
+    <hyperlink ref="B24" r:id="rId60"/>
+    <hyperlink ref="C24" r:id="rId61"/>
+    <hyperlink ref="B25" r:id="rId62"/>
+    <hyperlink ref="AJ25" r:id="rId63"/>
+    <hyperlink ref="B26" r:id="rId64"/>
+    <hyperlink ref="AJ26" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated dv1 questionnaire additional material
</commit_message>
<xml_diff>
--- a/resources/metadata_process_scripts/sources/catalog.xlsx
+++ b/resources/metadata_process_scripts/sources/catalog.xlsx
@@ -4683,10 +4683,10 @@
     <t>https://drive.google.com/file/d/1fXlb2vJfp_HOs4XP_3jaLYM7rTipGygO/view?usp=drive_link</t>
   </si>
   <si>
-    <t>https://drive.google.com/file/d/16loX2mvErVw_fzrBAYLX3uIwc_3FrwrA/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1i7-1KpYq-e7bkmqsACY_38sRtYwUpo1j/view?usp=sharing</t>
+    <t>https://drive.google.com/file/d/1jhkBFcruJil2f09xV1dYpjgQL-yqcbaj/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1bOYnYNkhHjpRO1WW0e2yDCSrKd4KwA-s/view?usp=drive_link</t>
   </si>
   <si>
     <t>002.AAAB.AAA.AY</t>

</xml_diff>

<commit_message>
fix mac tech report
</commit_message>
<xml_diff>
--- a/resources/metadata_process_scripts/sources/catalog.xlsx
+++ b/resources/metadata_process_scripts/sources/catalog.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11865" uniqueCount="2446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11862" uniqueCount="2446">
   <si>
     <t>ds:prjTitle</t>
   </si>
@@ -10137,15 +10137,6 @@
       <c r="AD25" t="s">
         <v>205</v>
       </c>
-      <c r="AI25" t="s">
-        <v>212</v>
-      </c>
-      <c r="AJ25" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="AK25" t="s">
-        <v>211</v>
-      </c>
       <c r="AL25" t="s">
         <v>219</v>
       </c>
@@ -10321,9 +10312,8 @@
     <hyperlink ref="B24" r:id="rId60"/>
     <hyperlink ref="C24" r:id="rId61"/>
     <hyperlink ref="B25" r:id="rId62"/>
-    <hyperlink ref="AJ25" r:id="rId63"/>
-    <hyperlink ref="B26" r:id="rId64"/>
-    <hyperlink ref="AJ26" r:id="rId65"/>
+    <hyperlink ref="B26" r:id="rId63"/>
+    <hyperlink ref="AJ26" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>